<commit_message>
Eintritte und Kiosk für Mutters Atelier und Das Licht
</commit_message>
<xml_diff>
--- a/Input/Verleiherabgaben.xlsx
+++ b/Input/Verleiherabgaben.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\R Packages\Kinoklub\Input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kinoklub\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11E9E70C-41CE-46A6-B6E4-08461F2D6364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44088841-7765-48E2-8939-AA06D953F0B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="14580" windowHeight="17370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Verleiherabgaben" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="158">
   <si>
     <t>Datum</t>
   </si>
@@ -509,6 +509,9 @@
   </si>
   <si>
     <t>1018.523</t>
+  </si>
+  <si>
+    <t>SC02.675</t>
   </si>
 </sst>
 </file>
@@ -627,7 +630,7 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{EB39806D-A340-4E6B-8E59-89A25516E3F2}"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="12">
     <dxf>
@@ -1091,21 +1094,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" customWidth="1"/>
-    <col min="2" max="2" width="12.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.453125" customWidth="1"/>
+    <col min="2" max="2" width="12.54296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.453125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="15.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="61.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="48.7109375" customWidth="1"/>
+    <col min="7" max="7" width="61.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="48.7265625" customWidth="1"/>
     <col min="9" max="9" width="43" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1131,7 +1134,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>45667</v>
       </c>
@@ -1152,7 +1155,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>45674</v>
       </c>
@@ -1174,7 +1177,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>45676</v>
       </c>
@@ -1196,7 +1199,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>45682</v>
       </c>
@@ -1218,7 +1221,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>45683</v>
       </c>
@@ -1240,7 +1243,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>45689</v>
       </c>
@@ -1262,7 +1265,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>45690</v>
       </c>
@@ -1284,7 +1287,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>45690</v>
       </c>
@@ -1306,7 +1309,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>45695</v>
       </c>
@@ -1328,7 +1331,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>45701</v>
       </c>
@@ -1350,7 +1353,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>45718</v>
       </c>
@@ -1371,7 +1374,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>45725</v>
       </c>
@@ -1392,7 +1395,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>45731</v>
       </c>
@@ -1413,7 +1416,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>45738</v>
       </c>
@@ -1434,7 +1437,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>45739</v>
       </c>
@@ -1455,7 +1458,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>45745</v>
       </c>
@@ -1476,7 +1479,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>45750</v>
       </c>
@@ -1497,7 +1500,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>45753</v>
       </c>
@@ -1518,7 +1521,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>45753</v>
       </c>
@@ -1539,7 +1542,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>45757</v>
       </c>
@@ -1560,7 +1563,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <v>45758</v>
       </c>
@@ -1581,7 +1584,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <v>45760</v>
       </c>
@@ -1602,7 +1605,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <v>45766</v>
       </c>
@@ -1623,11 +1626,14 @@
         <v>11</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <v>45773</v>
       </c>
       <c r="B25" s="8"/>
+      <c r="C25" s="1" t="s">
+        <v>157</v>
+      </c>
       <c r="D25" s="5">
         <v>150</v>
       </c>
@@ -1641,7 +1647,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <v>45781</v>
       </c>
@@ -1662,7 +1668,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <v>45781</v>
       </c>
@@ -1683,7 +1689,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <v>45787</v>
       </c>
@@ -1704,7 +1710,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <v>45793</v>
       </c>
@@ -1725,7 +1731,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <v>45795</v>
       </c>
@@ -1746,7 +1752,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>45801</v>
       </c>
@@ -1767,7 +1773,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <v>45807</v>
       </c>
@@ -1820,16 +1826,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2012A76-D168-4BE0-9450-2E40BA8CE7CD}">
   <dimension ref="A1:E36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="43.42578125" customWidth="1"/>
+    <col min="1" max="1" width="43.453125" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.81640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -1846,7 +1852,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>24</v>
       </c>
@@ -1863,7 +1869,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="3" t="s">
         <v>20</v>
       </c>
@@ -1880,7 +1886,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" ht="26" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
         <v>19</v>
       </c>
@@ -1897,7 +1903,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>52</v>
       </c>
@@ -1914,7 +1920,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>7</v>
       </c>
@@ -1931,7 +1937,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
         <v>10</v>
       </c>
@@ -1948,7 +1954,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
         <v>9</v>
       </c>
@@ -1965,7 +1971,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>11</v>
       </c>
@@ -1982,7 +1988,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="26" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>51</v>
       </c>
@@ -1999,7 +2005,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
         <v>14</v>
       </c>
@@ -2016,7 +2022,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>21</v>
       </c>
@@ -2033,7 +2039,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="26" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>18</v>
       </c>
@@ -2050,7 +2056,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
         <v>17</v>
       </c>
@@ -2067,7 +2073,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" ht="26" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
         <v>15</v>
       </c>
@@ -2084,7 +2090,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
         <v>13</v>
       </c>
@@ -2101,7 +2107,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" ht="26" x14ac:dyDescent="0.35">
       <c r="A17" s="4" t="s">
         <v>16</v>
       </c>
@@ -2118,7 +2124,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
         <v>8</v>
       </c>
@@ -2135,7 +2141,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
         <v>12</v>
       </c>
@@ -2152,7 +2158,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="3" t="s">
         <v>72</v>
       </c>
@@ -2169,7 +2175,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>74</v>
       </c>
@@ -2186,7 +2192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>77</v>
       </c>
@@ -2203,7 +2209,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>78</v>
       </c>
@@ -2220,7 +2226,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
         <v>85</v>
       </c>
@@ -2237,7 +2243,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="3" t="s">
         <v>87</v>
       </c>
@@ -2254,7 +2260,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" ht="26" x14ac:dyDescent="0.35">
       <c r="A26" s="3" t="s">
         <v>114</v>
       </c>
@@ -2271,7 +2277,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" ht="26" x14ac:dyDescent="0.35">
       <c r="A27" s="3" t="s">
         <v>152</v>
       </c>
@@ -2288,16 +2294,16 @@
         <v>155</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" s="9"/>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" s="9"/>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" s="9"/>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" s="9"/>
     </row>
   </sheetData>
@@ -2324,22 +2330,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB792523-3058-487E-914C-DA84AFB7228F}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" customWidth="1"/>
+    <col min="1" max="1" width="11.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>5</v>
       </c>

</xml_diff>